<commit_message>
level 3 custom cut formatted
old data can have different keys vs new data
</commit_message>
<xml_diff>
--- a/scratch/FormattedCutTableL3_template_md snippit.xlsx
+++ b/scratch/FormattedCutTableL3_template_md snippit.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Documents/UCET software/Data-Processing-Software/scratch/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4796E2E0-1A86-7941-9820-6AADC9530665}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AE9AD9A-92D7-F947-821A-4407555BE23C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20260" xr2:uid="{1837E1AF-DB18-D64C-9443-79C0B4F568AD}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="45">
   <si>
     <t>3R2</t>
   </si>
@@ -43,9 +43,6 @@
     <t>Metrics</t>
   </si>
   <si>
-    <t>units</t>
-  </si>
-  <si>
     <t>Operation</t>
   </si>
   <si>
@@ -100,9 +97,6 @@
     <t>initial_fuel_mass_1_lp</t>
   </si>
   <si>
-    <t>data_key</t>
-  </si>
-  <si>
     <t>stove_type/model</t>
   </si>
   <si>
@@ -118,9 +112,6 @@
     <t>4R2</t>
   </si>
   <si>
-    <t>data_type</t>
-  </si>
-  <si>
     <t>N</t>
   </si>
   <si>
@@ -157,7 +148,28 @@
     <t>lb/hr</t>
   </si>
   <si>
-    <t>sig_figs</t>
+    <t>units_1</t>
+  </si>
+  <si>
+    <t>sig_figs_1</t>
+  </si>
+  <si>
+    <t>data_type_1</t>
+  </si>
+  <si>
+    <t>data_key_1</t>
+  </si>
+  <si>
+    <t>fuel_dry_mass_1_L1</t>
+  </si>
+  <si>
+    <t>fuel_dry_mass_1_hp</t>
+  </si>
+  <si>
+    <t>fuel_dry_mass_1_mp</t>
+  </si>
+  <si>
+    <t>fuel_dry_mass_1_lp</t>
   </si>
 </sst>
 </file>
@@ -339,7 +351,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -355,7 +367,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -670,7 +681,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A22C1804-EB7C-BF43-9073-75DDFAF0ED4D}">
-  <dimension ref="B1:M36"/>
+  <dimension ref="B1:Q36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3.1640625" style="1" customWidth="1"/>
@@ -679,447 +690,625 @@
     <col min="5" max="6" width="4.5" style="1" customWidth="1"/>
     <col min="7" max="7" width="14.1640625" style="1" customWidth="1"/>
     <col min="8" max="8" width="23" style="1" customWidth="1"/>
-    <col min="9" max="10" width="6.5" style="2" customWidth="1"/>
-    <col min="11" max="12" width="6.5" style="3" customWidth="1"/>
-    <col min="13" max="13" width="10.83203125" style="2"/>
-    <col min="14" max="16384" width="10.83203125" style="1"/>
+    <col min="9" max="9" width="6.5" style="2" customWidth="1"/>
+    <col min="10" max="11" width="4.5" style="1" customWidth="1"/>
+    <col min="12" max="12" width="14.1640625" style="1" customWidth="1"/>
+    <col min="13" max="13" width="23" style="1" customWidth="1"/>
+    <col min="14" max="14" width="6.5" style="2" customWidth="1"/>
+    <col min="15" max="16" width="6.5" style="3" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" style="2"/>
+    <col min="18" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="3:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="3:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="H2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="3:17" x14ac:dyDescent="0.2">
+      <c r="C3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="3:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="H2" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="3:13" x14ac:dyDescent="0.2">
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="5"/>
+    </row>
+    <row r="4" spans="3:17" s="8" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+      <c r="C4" s="6" t="s">
         <v>3</v>
-      </c>
-      <c r="D3" s="5"/>
-    </row>
-    <row r="4" spans="3:13" s="8" customFormat="1" ht="14" x14ac:dyDescent="0.2">
-      <c r="C4" s="6" t="s">
-        <v>4</v>
       </c>
       <c r="D4" s="7"/>
       <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="10"/>
-      <c r="L4" s="10"/>
-      <c r="M4" s="9"/>
-    </row>
-    <row r="5" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="N4" s="9"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+      <c r="Q4" s="9"/>
+    </row>
+    <row r="5" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C5" s="11"/>
       <c r="D5" s="12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F5" s="1">
         <v>0</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="3:13" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+      <c r="K5" s="1">
+        <v>0</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C6" s="11"/>
       <c r="D6" s="12" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F6" s="1">
         <v>0</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="7" spans="3:13" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+      <c r="K6" s="1">
+        <v>0</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C7" s="11"/>
       <c r="D7" s="12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F7" s="1">
         <v>0</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8" spans="3:13" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+      <c r="K7" s="1">
+        <v>0</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C8" s="11"/>
       <c r="D8" s="12" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F8" s="1">
         <v>0</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="3:13" s="8" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+        <v>25</v>
+      </c>
+      <c r="K8" s="1">
+        <v>0</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="3:17" s="8" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C9" s="6" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D9" s="13"/>
       <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="9"/>
-    </row>
-    <row r="10" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="N9" s="9"/>
+      <c r="O9" s="10"/>
+      <c r="P9" s="10"/>
+      <c r="Q9" s="9"/>
+    </row>
+    <row r="10" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C10" s="11"/>
       <c r="D10" s="12" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="3:13" x14ac:dyDescent="0.2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C11" s="11"/>
       <c r="D11" s="12" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="3:13" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C12" s="11"/>
       <c r="D12" s="12" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="3:13" x14ac:dyDescent="0.2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C13" s="11"/>
       <c r="D13" s="12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="3:13" s="8" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="3:17" s="8" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C14" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D14" s="13"/>
       <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="9"/>
-    </row>
-    <row r="15" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="N14" s="9"/>
+      <c r="O14" s="10"/>
+      <c r="P14" s="10"/>
+      <c r="Q14" s="9"/>
+    </row>
+    <row r="15" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C15" s="11"/>
       <c r="D15" s="12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F15" s="1">
         <v>1</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H15" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="3:13" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+      <c r="K15" s="1">
+        <v>1</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C16" s="11"/>
       <c r="D16" s="12" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F16" s="1">
         <v>1</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H16" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" spans="3:13" x14ac:dyDescent="0.2">
+        <v>11</v>
+      </c>
+      <c r="K16" s="1">
+        <v>1</v>
+      </c>
+      <c r="L16" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C17" s="11"/>
       <c r="D17" s="12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F17" s="1">
         <v>1</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H17" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="3:13" x14ac:dyDescent="0.2">
+        <v>12</v>
+      </c>
+      <c r="K17" s="1">
+        <v>1</v>
+      </c>
+      <c r="L17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C18" s="11"/>
       <c r="D18" s="12" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F18" s="1">
         <v>1</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H18" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="3:13" x14ac:dyDescent="0.2">
+        <v>13</v>
+      </c>
+      <c r="K18" s="1">
+        <v>1</v>
+      </c>
+      <c r="L18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="M18" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C19" s="11"/>
       <c r="D19" s="12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F19" s="1">
         <v>1</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" spans="3:13" s="8" customFormat="1" ht="14" x14ac:dyDescent="0.2">
+        <v>15</v>
+      </c>
+      <c r="K19" s="1">
+        <v>1</v>
+      </c>
+      <c r="L19" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="M19" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="3:17" s="8" customFormat="1" ht="14" x14ac:dyDescent="0.2">
       <c r="C20" s="6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D20" s="13"/>
       <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
-      <c r="M20" s="9"/>
-    </row>
-    <row r="21" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="N20" s="9"/>
+      <c r="O20" s="10"/>
+      <c r="P20" s="10"/>
+      <c r="Q20" s="9"/>
+    </row>
+    <row r="21" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C21" s="11"/>
       <c r="D21" s="12" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H21" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22" spans="3:13" x14ac:dyDescent="0.2">
+        <v>16</v>
+      </c>
+      <c r="L21" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C22" s="11"/>
       <c r="D22" s="12" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H22" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="23" spans="3:13" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+      <c r="L22" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M22" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C23" s="11"/>
       <c r="D23" s="12" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H23" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="24" spans="3:13" x14ac:dyDescent="0.2">
+        <v>18</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M23" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C24" s="11"/>
       <c r="D24" s="12" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H24" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="25" spans="3:13" x14ac:dyDescent="0.2">
+        <v>19</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M24" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C25" s="11"/>
       <c r="D25" s="12" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="26" spans="3:13" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="26" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C26" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D26" s="13"/>
       <c r="E26" s="8"/>
-      <c r="F26" s="15"/>
       <c r="H26" s="8"/>
-    </row>
-    <row r="27" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="J26" s="8"/>
+      <c r="M26" s="8"/>
+    </row>
+    <row r="27" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C27" s="11"/>
       <c r="D27" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="F27" s="15"/>
+        <v>31</v>
+      </c>
       <c r="G27" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H27" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="28" spans="3:13" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="L27" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M27" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C28" s="11"/>
       <c r="D28" s="14" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E28" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="F28" s="15"/>
+        <v>31</v>
+      </c>
       <c r="G28" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H28" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="29" spans="3:13" x14ac:dyDescent="0.2">
+        <v>33</v>
+      </c>
+      <c r="J28" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="L28" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M28" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C29" s="11"/>
       <c r="D29" s="14" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E29" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="H29" t="s">
         <v>34</v>
       </c>
-      <c r="F29" s="15"/>
-      <c r="G29" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H29" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="30" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="J29" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="L29" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M29" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C30" s="11"/>
       <c r="D30" s="14" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E30" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="F30" s="15"/>
+        <v>31</v>
+      </c>
       <c r="G30" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H30" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="31" spans="3:13" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+      <c r="J30" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="L30" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C31" s="11"/>
       <c r="D31" s="14" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="32" spans="3:13" x14ac:dyDescent="0.2">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="32" spans="3:17" x14ac:dyDescent="0.2">
       <c r="C32" s="6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D32" s="13"/>
       <c r="E32" s="8"/>
-      <c r="F32" s="15"/>
       <c r="H32"/>
-    </row>
-    <row r="33" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="J32" s="8"/>
+      <c r="M32"/>
+    </row>
+    <row r="33" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C33" s="11"/>
       <c r="D33" s="14" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="F33" s="15"/>
+        <v>36</v>
+      </c>
       <c r="G33" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H33" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="34" spans="3:8" x14ac:dyDescent="0.2">
+        <v>32</v>
+      </c>
+      <c r="J33" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="L33" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M33" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="34" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C34" s="11"/>
       <c r="D34" s="14" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E34" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="F34" s="15"/>
+        <v>36</v>
+      </c>
       <c r="G34" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H34" t="s">
+        <v>33</v>
+      </c>
+      <c r="J34" s="8" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="35" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="L34" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M34" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C35" s="11"/>
       <c r="D35" s="14" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="F35" s="15"/>
+        <v>36</v>
+      </c>
       <c r="G35" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H35" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="36" spans="3:8" x14ac:dyDescent="0.2">
+        <v>34</v>
+      </c>
+      <c r="J35" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="L35" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M35" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="36" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C36" s="11"/>
       <c r="D36" s="14" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E36" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="F36" s="15"/>
+        <v>36</v>
+      </c>
       <c r="G36" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="H36" t="s">
-        <v>38</v>
+        <v>35</v>
+      </c>
+      <c r="J36" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="L36" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="M36" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>